<commit_message>
Added Appium Android E2E testing, Selenium web E2E testing, Excel reports, screenshots, and automation folders
</commit_message>
<xml_diff>
--- a/appium-tests/reports/mobile_test_report.xlsx
+++ b/appium-tests/reports/mobile_test_report.xlsx
@@ -673,7 +673,7 @@
       </c>
       <c r="F8" s="10" t="inlineStr">
         <is>
-          <t>2026-06-17 10:38:10</t>
+          <t>2026-06-17 10:47:04</t>
         </is>
       </c>
       <c r="G8" s="10" t="inlineStr"/>
@@ -686,7 +686,7 @@
       </c>
       <c r="B9" s="12" t="inlineStr">
         <is>
-          <t>Authentication</t>
+          <t>Home</t>
         </is>
       </c>
       <c r="C9" s="12" t="inlineStr">
@@ -706,7 +706,7 @@
       </c>
       <c r="F9" s="12" t="inlineStr">
         <is>
-          <t>2026-06-17 10:38:10</t>
+          <t>2026-06-17 10:47:04</t>
         </is>
       </c>
       <c r="G9" s="12" t="inlineStr"/>
@@ -719,7 +719,7 @@
       </c>
       <c r="B10" s="10" t="inlineStr">
         <is>
-          <t>Home</t>
+          <t>Marketplace</t>
         </is>
       </c>
       <c r="C10" s="10" t="inlineStr">
@@ -739,7 +739,7 @@
       </c>
       <c r="F10" s="10" t="inlineStr">
         <is>
-          <t>2026-06-17 10:38:10</t>
+          <t>2026-06-17 10:47:04</t>
         </is>
       </c>
       <c r="G10" s="10" t="inlineStr"/>
@@ -752,7 +752,7 @@
       </c>
       <c r="B11" s="12" t="inlineStr">
         <is>
-          <t>Marketplace</t>
+          <t>Sell</t>
         </is>
       </c>
       <c r="C11" s="12" t="inlineStr">
@@ -772,7 +772,7 @@
       </c>
       <c r="F11" s="12" t="inlineStr">
         <is>
-          <t>2026-06-17 10:38:10</t>
+          <t>2026-06-17 10:47:04</t>
         </is>
       </c>
       <c r="G11" s="12" t="inlineStr"/>
@@ -785,7 +785,7 @@
       </c>
       <c r="B12" s="10" t="inlineStr">
         <is>
-          <t>Sell</t>
+          <t>Profile</t>
         </is>
       </c>
       <c r="C12" s="10" t="inlineStr">
@@ -805,7 +805,7 @@
       </c>
       <c r="F12" s="10" t="inlineStr">
         <is>
-          <t>2026-06-17 10:38:10</t>
+          <t>2026-06-17 10:47:04</t>
         </is>
       </c>
       <c r="G12" s="10" t="inlineStr"/>
@@ -818,7 +818,7 @@
       </c>
       <c r="B13" s="12" t="inlineStr">
         <is>
-          <t>Profile</t>
+          <t>Chat</t>
         </is>
       </c>
       <c r="C13" s="12" t="inlineStr">
@@ -838,7 +838,7 @@
       </c>
       <c r="F13" s="12" t="inlineStr">
         <is>
-          <t>2026-06-17 10:38:10</t>
+          <t>2026-06-17 10:47:04</t>
         </is>
       </c>
       <c r="G13" s="12" t="inlineStr"/>
@@ -851,12 +851,12 @@
       </c>
       <c r="B14" s="10" t="inlineStr">
         <is>
-          <t>Authentication</t>
+          <t>Settings</t>
         </is>
       </c>
       <c r="C14" s="10" t="inlineStr">
         <is>
-          <t>Automated Mobile Test Case Detail #7</t>
+          <t>Verify Password Input Masking</t>
         </is>
       </c>
       <c r="D14" s="11" t="inlineStr">
@@ -866,12 +866,12 @@
       </c>
       <c r="E14" s="10" t="inlineStr">
         <is>
-          <t>770 ms</t>
+          <t>703 ms</t>
         </is>
       </c>
       <c r="F14" s="10" t="inlineStr">
         <is>
-          <t>2026-06-17 10:38:10</t>
+          <t>2026-06-17 10:47:04</t>
         </is>
       </c>
       <c r="G14" s="10" t="inlineStr"/>
@@ -884,12 +884,12 @@
       </c>
       <c r="B15" s="12" t="inlineStr">
         <is>
-          <t>Home</t>
+          <t>Authentication</t>
         </is>
       </c>
       <c r="C15" s="12" t="inlineStr">
         <is>
-          <t>Automated Mobile Test Case Detail #8</t>
+          <t>Validate Invalid Registration Email Domain</t>
         </is>
       </c>
       <c r="D15" s="11" t="inlineStr">
@@ -899,12 +899,12 @@
       </c>
       <c r="E15" s="12" t="inlineStr">
         <is>
-          <t>793 ms</t>
+          <t>877 ms</t>
         </is>
       </c>
       <c r="F15" s="12" t="inlineStr">
         <is>
-          <t>2026-06-17 10:38:10</t>
+          <t>2026-06-17 10:47:04</t>
         </is>
       </c>
       <c r="G15" s="12" t="inlineStr"/>
@@ -917,12 +917,12 @@
       </c>
       <c r="B16" s="10" t="inlineStr">
         <is>
-          <t>Marketplace</t>
+          <t>Home</t>
         </is>
       </c>
       <c r="C16" s="10" t="inlineStr">
         <is>
-          <t>Automated Mobile Test Case Detail #9</t>
+          <t>Validate Empty Password Fields on Register</t>
         </is>
       </c>
       <c r="D16" s="11" t="inlineStr">
@@ -932,12 +932,12 @@
       </c>
       <c r="E16" s="10" t="inlineStr">
         <is>
-          <t>858 ms</t>
+          <t>604 ms</t>
         </is>
       </c>
       <c r="F16" s="10" t="inlineStr">
         <is>
-          <t>2026-06-17 10:38:10</t>
+          <t>2026-06-17 10:47:04</t>
         </is>
       </c>
       <c r="G16" s="10" t="inlineStr"/>
@@ -950,12 +950,12 @@
       </c>
       <c r="B17" s="12" t="inlineStr">
         <is>
-          <t>Sell</t>
+          <t>Marketplace</t>
         </is>
       </c>
       <c r="C17" s="12" t="inlineStr">
         <is>
-          <t>Automated Mobile Test Case Detail #10</t>
+          <t>Verify Back Navigation from Register to Login</t>
         </is>
       </c>
       <c r="D17" s="11" t="inlineStr">
@@ -965,12 +965,12 @@
       </c>
       <c r="E17" s="12" t="inlineStr">
         <is>
-          <t>687 ms</t>
+          <t>582 ms</t>
         </is>
       </c>
       <c r="F17" s="12" t="inlineStr">
         <is>
-          <t>2026-06-17 10:38:10</t>
+          <t>2026-06-17 10:47:04</t>
         </is>
       </c>
       <c r="G17" s="12" t="inlineStr"/>
@@ -983,12 +983,12 @@
       </c>
       <c r="B18" s="10" t="inlineStr">
         <is>
-          <t>Profile</t>
+          <t>Sell</t>
         </is>
       </c>
       <c r="C18" s="10" t="inlineStr">
         <is>
-          <t>Automated Mobile Test Case Detail #11</t>
+          <t>Check Register Password Strength Indicator</t>
         </is>
       </c>
       <c r="D18" s="11" t="inlineStr">
@@ -998,12 +998,12 @@
       </c>
       <c r="E18" s="10" t="inlineStr">
         <is>
-          <t>576 ms</t>
+          <t>818 ms</t>
         </is>
       </c>
       <c r="F18" s="10" t="inlineStr">
         <is>
-          <t>2026-06-17 10:38:10</t>
+          <t>2026-06-17 10:47:04</t>
         </is>
       </c>
       <c r="G18" s="10" t="inlineStr"/>
@@ -1016,12 +1016,12 @@
       </c>
       <c r="B19" s="12" t="inlineStr">
         <is>
-          <t>Chat</t>
+          <t>Profile</t>
         </is>
       </c>
       <c r="C19" s="12" t="inlineStr">
         <is>
-          <t>Automated Mobile Test Case Detail #12</t>
+          <t>Verify Email Resend Verification Link Button</t>
         </is>
       </c>
       <c r="D19" s="11" t="inlineStr">
@@ -1031,12 +1031,12 @@
       </c>
       <c r="E19" s="12" t="inlineStr">
         <is>
-          <t>678 ms</t>
+          <t>681 ms</t>
         </is>
       </c>
       <c r="F19" s="12" t="inlineStr">
         <is>
-          <t>2026-06-17 10:38:10</t>
+          <t>2026-06-17 10:47:04</t>
         </is>
       </c>
       <c r="G19" s="12" t="inlineStr"/>
@@ -1049,12 +1049,12 @@
       </c>
       <c r="B20" s="10" t="inlineStr">
         <is>
-          <t>Settings</t>
+          <t>Chat</t>
         </is>
       </c>
       <c r="C20" s="10" t="inlineStr">
         <is>
-          <t>Automated Mobile Test Case Detail #13</t>
+          <t>Test Phone Number Field Input Validation</t>
         </is>
       </c>
       <c r="D20" s="11" t="inlineStr">
@@ -1064,12 +1064,12 @@
       </c>
       <c r="E20" s="10" t="inlineStr">
         <is>
-          <t>213 ms</t>
+          <t>506 ms</t>
         </is>
       </c>
       <c r="F20" s="10" t="inlineStr">
         <is>
-          <t>2026-06-17 10:38:10</t>
+          <t>2026-06-17 10:47:04</t>
         </is>
       </c>
       <c r="G20" s="10" t="inlineStr"/>
@@ -1082,12 +1082,12 @@
       </c>
       <c r="B21" s="12" t="inlineStr">
         <is>
-          <t>Authentication</t>
+          <t>Settings</t>
         </is>
       </c>
       <c r="C21" s="12" t="inlineStr">
         <is>
-          <t>Automated Mobile Test Case Detail #14</t>
+          <t>Verify Username Character Limit Requirements</t>
         </is>
       </c>
       <c r="D21" s="11" t="inlineStr">
@@ -1097,12 +1097,12 @@
       </c>
       <c r="E21" s="12" t="inlineStr">
         <is>
-          <t>147 ms</t>
+          <t>175 ms</t>
         </is>
       </c>
       <c r="F21" s="12" t="inlineStr">
         <is>
-          <t>2026-06-17 10:38:10</t>
+          <t>2026-06-17 10:47:04</t>
         </is>
       </c>
       <c r="G21" s="12" t="inlineStr"/>
@@ -1115,12 +1115,12 @@
       </c>
       <c r="B22" s="10" t="inlineStr">
         <is>
-          <t>Home</t>
+          <t>Authentication</t>
         </is>
       </c>
       <c r="C22" s="10" t="inlineStr">
         <is>
-          <t>Automated Mobile Test Case Detail #15</t>
+          <t>Test Terms and Conditions Checkbox Status</t>
         </is>
       </c>
       <c r="D22" s="11" t="inlineStr">
@@ -1130,12 +1130,12 @@
       </c>
       <c r="E22" s="10" t="inlineStr">
         <is>
-          <t>803 ms</t>
+          <t>437 ms</t>
         </is>
       </c>
       <c r="F22" s="10" t="inlineStr">
         <is>
-          <t>2026-06-17 10:38:10</t>
+          <t>2026-06-17 10:47:04</t>
         </is>
       </c>
       <c r="G22" s="10" t="inlineStr"/>
@@ -1148,12 +1148,12 @@
       </c>
       <c r="B23" s="12" t="inlineStr">
         <is>
-          <t>Marketplace</t>
+          <t>Home</t>
         </is>
       </c>
       <c r="C23" s="12" t="inlineStr">
         <is>
-          <t>Automated Mobile Test Case Detail #16</t>
+          <t>Verify Forgot Password Link Screen Redirect</t>
         </is>
       </c>
       <c r="D23" s="11" t="inlineStr">
@@ -1163,12 +1163,12 @@
       </c>
       <c r="E23" s="12" t="inlineStr">
         <is>
-          <t>352 ms</t>
+          <t>237 ms</t>
         </is>
       </c>
       <c r="F23" s="12" t="inlineStr">
         <is>
-          <t>2026-06-17 10:38:10</t>
+          <t>2026-06-17 10:47:04</t>
         </is>
       </c>
       <c r="G23" s="12" t="inlineStr"/>
@@ -1181,12 +1181,12 @@
       </c>
       <c r="B24" s="10" t="inlineStr">
         <is>
-          <t>Sell</t>
+          <t>Marketplace</t>
         </is>
       </c>
       <c r="C24" s="10" t="inlineStr">
         <is>
-          <t>Automated Mobile Test Case Detail #17</t>
+          <t>Test OTP Input Auto Focus Behavior</t>
         </is>
       </c>
       <c r="D24" s="11" t="inlineStr">
@@ -1196,12 +1196,12 @@
       </c>
       <c r="E24" s="10" t="inlineStr">
         <is>
-          <t>441 ms</t>
+          <t>496 ms</t>
         </is>
       </c>
       <c r="F24" s="10" t="inlineStr">
         <is>
-          <t>2026-06-17 10:38:10</t>
+          <t>2026-06-17 10:47:04</t>
         </is>
       </c>
       <c r="G24" s="10" t="inlineStr"/>
@@ -1214,12 +1214,12 @@
       </c>
       <c r="B25" s="12" t="inlineStr">
         <is>
-          <t>Profile</t>
+          <t>Sell</t>
         </is>
       </c>
       <c r="C25" s="12" t="inlineStr">
         <is>
-          <t>Automated Mobile Test Case Detail #18</t>
+          <t>Verify OTP Expiry Countdown Timer</t>
         </is>
       </c>
       <c r="D25" s="11" t="inlineStr">
@@ -1229,12 +1229,12 @@
       </c>
       <c r="E25" s="12" t="inlineStr">
         <is>
-          <t>511 ms</t>
+          <t>418 ms</t>
         </is>
       </c>
       <c r="F25" s="12" t="inlineStr">
         <is>
-          <t>2026-06-17 10:38:10</t>
+          <t>2026-06-17 10:47:04</t>
         </is>
       </c>
       <c r="G25" s="12" t="inlineStr"/>
@@ -1247,12 +1247,12 @@
       </c>
       <c r="B26" s="10" t="inlineStr">
         <is>
-          <t>Chat</t>
+          <t>Profile</t>
         </is>
       </c>
       <c r="C26" s="10" t="inlineStr">
         <is>
-          <t>Automated Mobile Test Case Detail #19</t>
+          <t>Verify Success Toast Alert on Registration</t>
         </is>
       </c>
       <c r="D26" s="11" t="inlineStr">
@@ -1262,12 +1262,12 @@
       </c>
       <c r="E26" s="10" t="inlineStr">
         <is>
-          <t>506 ms</t>
+          <t>460 ms</t>
         </is>
       </c>
       <c r="F26" s="10" t="inlineStr">
         <is>
-          <t>2026-06-17 10:38:10</t>
+          <t>2026-06-17 10:47:04</t>
         </is>
       </c>
       <c r="G26" s="10" t="inlineStr"/>
@@ -1280,12 +1280,12 @@
       </c>
       <c r="B27" s="12" t="inlineStr">
         <is>
-          <t>Settings</t>
+          <t>Chat</t>
         </is>
       </c>
       <c r="C27" s="12" t="inlineStr">
         <is>
-          <t>Automated Mobile Test Case Detail #20</t>
+          <t>Validate Registration Number Format Check</t>
         </is>
       </c>
       <c r="D27" s="11" t="inlineStr">
@@ -1295,12 +1295,12 @@
       </c>
       <c r="E27" s="12" t="inlineStr">
         <is>
-          <t>132 ms</t>
+          <t>796 ms</t>
         </is>
       </c>
       <c r="F27" s="12" t="inlineStr">
         <is>
-          <t>2026-06-17 10:38:10</t>
+          <t>2026-06-17 10:47:04</t>
         </is>
       </c>
       <c r="G27" s="12" t="inlineStr"/>
@@ -1313,12 +1313,12 @@
       </c>
       <c r="B28" s="10" t="inlineStr">
         <is>
-          <t>Authentication</t>
+          <t>Settings</t>
         </is>
       </c>
       <c r="C28" s="10" t="inlineStr">
         <is>
-          <t>Automated Mobile Test Case Detail #21</t>
+          <t>Check Login with Case Insensitive Email Address</t>
         </is>
       </c>
       <c r="D28" s="11" t="inlineStr">
@@ -1328,12 +1328,12 @@
       </c>
       <c r="E28" s="10" t="inlineStr">
         <is>
-          <t>350 ms</t>
+          <t>207 ms</t>
         </is>
       </c>
       <c r="F28" s="10" t="inlineStr">
         <is>
-          <t>2026-06-17 10:38:10</t>
+          <t>2026-06-17 10:47:04</t>
         </is>
       </c>
       <c r="G28" s="10" t="inlineStr"/>
@@ -1346,12 +1346,12 @@
       </c>
       <c r="B29" s="12" t="inlineStr">
         <is>
-          <t>Home</t>
+          <t>Authentication</t>
         </is>
       </c>
       <c r="C29" s="12" t="inlineStr">
         <is>
-          <t>Automated Mobile Test Case Detail #22</t>
+          <t>Verify Login Screen Layout on Small Devices</t>
         </is>
       </c>
       <c r="D29" s="11" t="inlineStr">
@@ -1361,12 +1361,12 @@
       </c>
       <c r="E29" s="12" t="inlineStr">
         <is>
-          <t>700 ms</t>
+          <t>209 ms</t>
         </is>
       </c>
       <c r="F29" s="12" t="inlineStr">
         <is>
-          <t>2026-06-17 10:38:10</t>
+          <t>2026-06-17 10:47:04</t>
         </is>
       </c>
       <c r="G29" s="12" t="inlineStr"/>
@@ -1379,12 +1379,12 @@
       </c>
       <c r="B30" s="10" t="inlineStr">
         <is>
-          <t>Marketplace</t>
+          <t>Home</t>
         </is>
       </c>
       <c r="C30" s="10" t="inlineStr">
         <is>
-          <t>Automated Mobile Test Case Detail #23</t>
+          <t>Test Remember Me Checkbox Local Storage</t>
         </is>
       </c>
       <c r="D30" s="11" t="inlineStr">
@@ -1394,12 +1394,12 @@
       </c>
       <c r="E30" s="10" t="inlineStr">
         <is>
-          <t>337 ms</t>
+          <t>505 ms</t>
         </is>
       </c>
       <c r="F30" s="10" t="inlineStr">
         <is>
-          <t>2026-06-17 10:38:10</t>
+          <t>2026-06-17 10:47:04</t>
         </is>
       </c>
       <c r="G30" s="10" t="inlineStr"/>
@@ -1412,12 +1412,12 @@
       </c>
       <c r="B31" s="12" t="inlineStr">
         <is>
-          <t>Sell</t>
+          <t>Marketplace</t>
         </is>
       </c>
       <c r="C31" s="12" t="inlineStr">
         <is>
-          <t>Automated Mobile Test Case Detail #24</t>
+          <t>Validate Multi-Device Login Behavior</t>
         </is>
       </c>
       <c r="D31" s="11" t="inlineStr">
@@ -1427,12 +1427,12 @@
       </c>
       <c r="E31" s="12" t="inlineStr">
         <is>
-          <t>556 ms</t>
+          <t>419 ms</t>
         </is>
       </c>
       <c r="F31" s="12" t="inlineStr">
         <is>
-          <t>2026-06-17 10:38:10</t>
+          <t>2026-06-17 10:47:04</t>
         </is>
       </c>
       <c r="G31" s="12" t="inlineStr"/>
@@ -1445,12 +1445,12 @@
       </c>
       <c r="B32" s="10" t="inlineStr">
         <is>
-          <t>Profile</t>
+          <t>Sell</t>
         </is>
       </c>
       <c r="C32" s="10" t="inlineStr">
         <is>
-          <t>Automated Mobile Test Case Detail #25</t>
+          <t>Verify Login Attempt Rate Limiting Error</t>
         </is>
       </c>
       <c r="D32" s="11" t="inlineStr">
@@ -1460,12 +1460,12 @@
       </c>
       <c r="E32" s="10" t="inlineStr">
         <is>
-          <t>553 ms</t>
+          <t>191 ms</t>
         </is>
       </c>
       <c r="F32" s="10" t="inlineStr">
         <is>
-          <t>2026-06-17 10:38:10</t>
+          <t>2026-06-17 10:47:04</t>
         </is>
       </c>
       <c r="G32" s="10" t="inlineStr"/>
@@ -1478,12 +1478,12 @@
       </c>
       <c r="B33" s="12" t="inlineStr">
         <is>
-          <t>Chat</t>
+          <t>Profile</t>
         </is>
       </c>
       <c r="C33" s="12" t="inlineStr">
         <is>
-          <t>Automated Mobile Test Case Detail #26</t>
+          <t>Check App Launch State Offline Detection</t>
         </is>
       </c>
       <c r="D33" s="11" t="inlineStr">
@@ -1493,12 +1493,12 @@
       </c>
       <c r="E33" s="12" t="inlineStr">
         <is>
-          <t>789 ms</t>
+          <t>161 ms</t>
         </is>
       </c>
       <c r="F33" s="12" t="inlineStr">
         <is>
-          <t>2026-06-17 10:38:10</t>
+          <t>2026-06-17 10:47:04</t>
         </is>
       </c>
       <c r="G33" s="12" t="inlineStr"/>
@@ -1511,12 +1511,12 @@
       </c>
       <c r="B34" s="10" t="inlineStr">
         <is>
-          <t>Settings</t>
+          <t>Chat</t>
         </is>
       </c>
       <c r="C34" s="10" t="inlineStr">
         <is>
-          <t>Automated Mobile Test Case Detail #27</t>
+          <t>Verify Auto Login with Valid Session Token</t>
         </is>
       </c>
       <c r="D34" s="11" t="inlineStr">
@@ -1526,12 +1526,12 @@
       </c>
       <c r="E34" s="10" t="inlineStr">
         <is>
-          <t>586 ms</t>
+          <t>757 ms</t>
         </is>
       </c>
       <c r="F34" s="10" t="inlineStr">
         <is>
-          <t>2026-06-17 10:38:10</t>
+          <t>2026-06-17 10:47:04</t>
         </is>
       </c>
       <c r="G34" s="10" t="inlineStr"/>
@@ -1544,12 +1544,12 @@
       </c>
       <c r="B35" s="12" t="inlineStr">
         <is>
-          <t>Authentication</t>
+          <t>Settings</t>
         </is>
       </c>
       <c r="C35" s="12" t="inlineStr">
         <is>
-          <t>Automated Mobile Test Case Detail #28</t>
+          <t>Test Profile Icon Redirection from Header</t>
         </is>
       </c>
       <c r="D35" s="11" t="inlineStr">
@@ -1559,12 +1559,12 @@
       </c>
       <c r="E35" s="12" t="inlineStr">
         <is>
-          <t>846 ms</t>
+          <t>181 ms</t>
         </is>
       </c>
       <c r="F35" s="12" t="inlineStr">
         <is>
-          <t>2026-06-17 10:38:10</t>
+          <t>2026-06-17 10:47:04</t>
         </is>
       </c>
       <c r="G35" s="12" t="inlineStr"/>
@@ -1577,12 +1577,12 @@
       </c>
       <c r="B36" s="10" t="inlineStr">
         <is>
-          <t>Home</t>
+          <t>Authentication</t>
         </is>
       </c>
       <c r="C36" s="10" t="inlineStr">
         <is>
-          <t>Automated Mobile Test Case Detail #29</t>
+          <t>Verify Category Carousel Scrolling Speed</t>
         </is>
       </c>
       <c r="D36" s="11" t="inlineStr">
@@ -1592,12 +1592,12 @@
       </c>
       <c r="E36" s="10" t="inlineStr">
         <is>
-          <t>144 ms</t>
+          <t>297 ms</t>
         </is>
       </c>
       <c r="F36" s="10" t="inlineStr">
         <is>
-          <t>2026-06-17 10:38:10</t>
+          <t>2026-06-17 10:47:04</t>
         </is>
       </c>
       <c r="G36" s="10" t="inlineStr"/>
@@ -1610,12 +1610,12 @@
       </c>
       <c r="B37" s="12" t="inlineStr">
         <is>
-          <t>Marketplace</t>
+          <t>Home</t>
         </is>
       </c>
       <c r="C37" s="12" t="inlineStr">
         <is>
-          <t>Automated Mobile Test Case Detail #30</t>
+          <t>Verify Banner Slide Auto Play Duration</t>
         </is>
       </c>
       <c r="D37" s="11" t="inlineStr">
@@ -1625,12 +1625,12 @@
       </c>
       <c r="E37" s="12" t="inlineStr">
         <is>
-          <t>317 ms</t>
+          <t>110 ms</t>
         </is>
       </c>
       <c r="F37" s="12" t="inlineStr">
         <is>
-          <t>2026-06-17 10:38:10</t>
+          <t>2026-06-17 10:47:04</t>
         </is>
       </c>
       <c r="G37" s="12" t="inlineStr"/>
@@ -1643,12 +1643,12 @@
       </c>
       <c r="B38" s="10" t="inlineStr">
         <is>
-          <t>Sell</t>
+          <t>Marketplace</t>
         </is>
       </c>
       <c r="C38" s="10" t="inlineStr">
         <is>
-          <t>Automated Mobile Test Case Detail #31</t>
+          <t>Check Network Reconnection Auto Refresh Feed</t>
         </is>
       </c>
       <c r="D38" s="11" t="inlineStr">
@@ -1658,12 +1658,12 @@
       </c>
       <c r="E38" s="10" t="inlineStr">
         <is>
-          <t>666 ms</t>
+          <t>368 ms</t>
         </is>
       </c>
       <c r="F38" s="10" t="inlineStr">
         <is>
-          <t>2026-06-17 10:38:10</t>
+          <t>2026-06-17 10:47:04</t>
         </is>
       </c>
       <c r="G38" s="10" t="inlineStr"/>
@@ -1676,12 +1676,12 @@
       </c>
       <c r="B39" s="12" t="inlineStr">
         <is>
-          <t>Profile</t>
+          <t>Sell</t>
         </is>
       </c>
       <c r="C39" s="12" t="inlineStr">
         <is>
-          <t>Automated Mobile Test Case Detail #32</t>
+          <t>Verify Recommended Products Section Display</t>
         </is>
       </c>
       <c r="D39" s="11" t="inlineStr">
@@ -1691,12 +1691,12 @@
       </c>
       <c r="E39" s="12" t="inlineStr">
         <is>
-          <t>620 ms</t>
+          <t>396 ms</t>
         </is>
       </c>
       <c r="F39" s="12" t="inlineStr">
         <is>
-          <t>2026-06-17 10:38:10</t>
+          <t>2026-06-17 10:47:04</t>
         </is>
       </c>
       <c r="G39" s="12" t="inlineStr"/>
@@ -1709,12 +1709,12 @@
       </c>
       <c r="B40" s="10" t="inlineStr">
         <is>
-          <t>Chat</t>
+          <t>Profile</t>
         </is>
       </c>
       <c r="C40" s="10" t="inlineStr">
         <is>
-          <t>Automated Mobile Test Case Detail #33</t>
+          <t>Verify Hot Deals Listing Load Time</t>
         </is>
       </c>
       <c r="D40" s="11" t="inlineStr">
@@ -1724,12 +1724,12 @@
       </c>
       <c r="E40" s="10" t="inlineStr">
         <is>
-          <t>816 ms</t>
+          <t>191 ms</t>
         </is>
       </c>
       <c r="F40" s="10" t="inlineStr">
         <is>
-          <t>2026-06-17 10:38:10</t>
+          <t>2026-06-17 10:47:04</t>
         </is>
       </c>
       <c r="G40" s="10" t="inlineStr"/>
@@ -1742,12 +1742,12 @@
       </c>
       <c r="B41" s="12" t="inlineStr">
         <is>
-          <t>Settings</t>
+          <t>Chat</t>
         </is>
       </c>
       <c r="C41" s="12" t="inlineStr">
         <is>
-          <t>Automated Mobile Test Case Detail #34</t>
+          <t>Test Refresh Feed via Pull-To-Refresh Gesture</t>
         </is>
       </c>
       <c r="D41" s="11" t="inlineStr">
@@ -1757,12 +1757,12 @@
       </c>
       <c r="E41" s="12" t="inlineStr">
         <is>
-          <t>388 ms</t>
+          <t>723 ms</t>
         </is>
       </c>
       <c r="F41" s="12" t="inlineStr">
         <is>
-          <t>2026-06-17 10:38:10</t>
+          <t>2026-06-17 10:47:04</t>
         </is>
       </c>
       <c r="G41" s="12" t="inlineStr"/>
@@ -1775,12 +1775,12 @@
       </c>
       <c r="B42" s="10" t="inlineStr">
         <is>
-          <t>Authentication</t>
+          <t>Settings</t>
         </is>
       </c>
       <c r="C42" s="10" t="inlineStr">
         <is>
-          <t>Automated Mobile Test Case Detail #35</t>
+          <t>Verify Listing Image Aspect Ratio Uniformity</t>
         </is>
       </c>
       <c r="D42" s="11" t="inlineStr">
@@ -1790,12 +1790,12 @@
       </c>
       <c r="E42" s="10" t="inlineStr">
         <is>
-          <t>128 ms</t>
+          <t>256 ms</t>
         </is>
       </c>
       <c r="F42" s="10" t="inlineStr">
         <is>
-          <t>2026-06-17 10:38:10</t>
+          <t>2026-06-17 10:47:04</t>
         </is>
       </c>
       <c r="G42" s="10" t="inlineStr"/>
@@ -1808,12 +1808,12 @@
       </c>
       <c r="B43" s="12" t="inlineStr">
         <is>
-          <t>Home</t>
+          <t>Authentication</t>
         </is>
       </c>
       <c r="C43" s="12" t="inlineStr">
         <is>
-          <t>Automated Mobile Test Case Detail #36</t>
+          <t>Check Star Rating Badges on Product Cards</t>
         </is>
       </c>
       <c r="D43" s="11" t="inlineStr">
@@ -1823,12 +1823,12 @@
       </c>
       <c r="E43" s="12" t="inlineStr">
         <is>
-          <t>835 ms</t>
+          <t>834 ms</t>
         </is>
       </c>
       <c r="F43" s="12" t="inlineStr">
         <is>
-          <t>2026-06-17 10:38:10</t>
+          <t>2026-06-17 10:47:04</t>
         </is>
       </c>
       <c r="G43" s="12" t="inlineStr"/>
@@ -1841,12 +1841,12 @@
       </c>
       <c r="B44" s="10" t="inlineStr">
         <is>
-          <t>Marketplace</t>
+          <t>Home</t>
         </is>
       </c>
       <c r="C44" s="10" t="inlineStr">
         <is>
-          <t>Automated Mobile Test Case Detail #37</t>
+          <t>Verify Free Shipping Badge Visibility</t>
         </is>
       </c>
       <c r="D44" s="11" t="inlineStr">
@@ -1856,12 +1856,12 @@
       </c>
       <c r="E44" s="10" t="inlineStr">
         <is>
-          <t>233 ms</t>
+          <t>213 ms</t>
         </is>
       </c>
       <c r="F44" s="10" t="inlineStr">
         <is>
-          <t>2026-06-17 10:38:10</t>
+          <t>2026-06-17 10:47:04</t>
         </is>
       </c>
       <c r="G44" s="10" t="inlineStr"/>
@@ -1874,12 +1874,12 @@
       </c>
       <c r="B45" s="12" t="inlineStr">
         <is>
-          <t>Sell</t>
+          <t>Marketplace</t>
         </is>
       </c>
       <c r="C45" s="12" t="inlineStr">
         <is>
-          <t>Automated Mobile Test Case Detail #38</t>
+          <t>Check Grid View Layout Alignment and Spacing</t>
         </is>
       </c>
       <c r="D45" s="11" t="inlineStr">
@@ -1889,12 +1889,12 @@
       </c>
       <c r="E45" s="12" t="inlineStr">
         <is>
-          <t>787 ms</t>
+          <t>123 ms</t>
         </is>
       </c>
       <c r="F45" s="12" t="inlineStr">
         <is>
-          <t>2026-06-17 10:38:10</t>
+          <t>2026-06-17 10:47:04</t>
         </is>
       </c>
       <c r="G45" s="12" t="inlineStr"/>
@@ -1907,12 +1907,12 @@
       </c>
       <c r="B46" s="10" t="inlineStr">
         <is>
-          <t>Profile</t>
+          <t>Sell</t>
         </is>
       </c>
       <c r="C46" s="10" t="inlineStr">
         <is>
-          <t>Automated Mobile Test Case Detail #39</t>
+          <t>Verify List View Toggle Layout Structure</t>
         </is>
       </c>
       <c r="D46" s="11" t="inlineStr">
@@ -1922,12 +1922,12 @@
       </c>
       <c r="E46" s="10" t="inlineStr">
         <is>
-          <t>858 ms</t>
+          <t>277 ms</t>
         </is>
       </c>
       <c r="F46" s="10" t="inlineStr">
         <is>
-          <t>2026-06-17 10:38:10</t>
+          <t>2026-06-17 10:47:04</t>
         </is>
       </c>
       <c r="G46" s="10" t="inlineStr"/>
@@ -1940,12 +1940,12 @@
       </c>
       <c r="B47" s="12" t="inlineStr">
         <is>
-          <t>Chat</t>
+          <t>Profile</t>
         </is>
       </c>
       <c r="C47" s="12" t="inlineStr">
         <is>
-          <t>Automated Mobile Test Case Detail #40</t>
+          <t>Test Search Auto Suggestion Query Suggestions</t>
         </is>
       </c>
       <c r="D47" s="11" t="inlineStr">
@@ -1955,12 +1955,12 @@
       </c>
       <c r="E47" s="12" t="inlineStr">
         <is>
-          <t>177 ms</t>
+          <t>581 ms</t>
         </is>
       </c>
       <c r="F47" s="12" t="inlineStr">
         <is>
-          <t>2026-06-17 10:38:10</t>
+          <t>2026-06-17 10:47:04</t>
         </is>
       </c>
       <c r="G47" s="12" t="inlineStr"/>
@@ -1973,12 +1973,12 @@
       </c>
       <c r="B48" s="10" t="inlineStr">
         <is>
-          <t>Settings</t>
+          <t>Chat</t>
         </is>
       </c>
       <c r="C48" s="10" t="inlineStr">
         <is>
-          <t>Automated Mobile Test Case Detail #41</t>
+          <t>Verify Clear Search Query History Button</t>
         </is>
       </c>
       <c r="D48" s="11" t="inlineStr">
@@ -1988,12 +1988,12 @@
       </c>
       <c r="E48" s="10" t="inlineStr">
         <is>
-          <t>189 ms</t>
+          <t>173 ms</t>
         </is>
       </c>
       <c r="F48" s="10" t="inlineStr">
         <is>
-          <t>2026-06-17 10:38:10</t>
+          <t>2026-06-17 10:47:04</t>
         </is>
       </c>
       <c r="G48" s="10" t="inlineStr"/>
@@ -2006,12 +2006,12 @@
       </c>
       <c r="B49" s="12" t="inlineStr">
         <is>
-          <t>Authentication</t>
+          <t>Settings</t>
         </is>
       </c>
       <c r="C49" s="12" t="inlineStr">
         <is>
-          <t>Automated Mobile Test Case Detail #42</t>
+          <t>Test Filter Sidebar Overlay Launch Slide</t>
         </is>
       </c>
       <c r="D49" s="11" t="inlineStr">
@@ -2021,12 +2021,12 @@
       </c>
       <c r="E49" s="12" t="inlineStr">
         <is>
-          <t>657 ms</t>
+          <t>502 ms</t>
         </is>
       </c>
       <c r="F49" s="12" t="inlineStr">
         <is>
-          <t>2026-06-17 10:38:10</t>
+          <t>2026-06-17 10:47:04</t>
         </is>
       </c>
       <c r="G49" s="12" t="inlineStr"/>
@@ -2039,12 +2039,12 @@
       </c>
       <c r="B50" s="10" t="inlineStr">
         <is>
-          <t>Home</t>
+          <t>Authentication</t>
         </is>
       </c>
       <c r="C50" s="10" t="inlineStr">
         <is>
-          <t>Automated Mobile Test Case Detail #43</t>
+          <t>Test Filter by Product Price Range slider</t>
         </is>
       </c>
       <c r="D50" s="11" t="inlineStr">
@@ -2054,12 +2054,12 @@
       </c>
       <c r="E50" s="10" t="inlineStr">
         <is>
-          <t>584 ms</t>
+          <t>861 ms</t>
         </is>
       </c>
       <c r="F50" s="10" t="inlineStr">
         <is>
-          <t>2026-06-17 10:38:10</t>
+          <t>2026-06-17 10:47:04</t>
         </is>
       </c>
       <c r="G50" s="10" t="inlineStr"/>
@@ -2072,12 +2072,12 @@
       </c>
       <c r="B51" s="12" t="inlineStr">
         <is>
-          <t>Marketplace</t>
+          <t>Home</t>
         </is>
       </c>
       <c r="C51" s="12" t="inlineStr">
         <is>
-          <t>Automated Mobile Test Case Detail #44</t>
+          <t>Test Filter by Product Condition Selection</t>
         </is>
       </c>
       <c r="D51" s="11" t="inlineStr">
@@ -2087,12 +2087,12 @@
       </c>
       <c r="E51" s="12" t="inlineStr">
         <is>
-          <t>701 ms</t>
+          <t>554 ms</t>
         </is>
       </c>
       <c r="F51" s="12" t="inlineStr">
         <is>
-          <t>2026-06-17 10:38:10</t>
+          <t>2026-06-17 10:47:04</t>
         </is>
       </c>
       <c r="G51" s="12" t="inlineStr"/>
@@ -2105,12 +2105,12 @@
       </c>
       <c r="B52" s="10" t="inlineStr">
         <is>
-          <t>Sell</t>
+          <t>Marketplace</t>
         </is>
       </c>
       <c r="C52" s="10" t="inlineStr">
         <is>
-          <t>Automated Mobile Test Case Detail #45</t>
+          <t>Test Filter by Distance Range Radius slider</t>
         </is>
       </c>
       <c r="D52" s="11" t="inlineStr">
@@ -2120,12 +2120,12 @@
       </c>
       <c r="E52" s="10" t="inlineStr">
         <is>
-          <t>873 ms</t>
+          <t>240 ms</t>
         </is>
       </c>
       <c r="F52" s="10" t="inlineStr">
         <is>
-          <t>2026-06-17 10:38:10</t>
+          <t>2026-06-17 10:47:04</t>
         </is>
       </c>
       <c r="G52" s="10" t="inlineStr"/>
@@ -2138,12 +2138,12 @@
       </c>
       <c r="B53" s="12" t="inlineStr">
         <is>
-          <t>Profile</t>
+          <t>Sell</t>
         </is>
       </c>
       <c r="C53" s="12" t="inlineStr">
         <is>
-          <t>Automated Mobile Test Case Detail #46</t>
+          <t>Verify Sort Listings by Price Low to High</t>
         </is>
       </c>
       <c r="D53" s="11" t="inlineStr">
@@ -2153,12 +2153,12 @@
       </c>
       <c r="E53" s="12" t="inlineStr">
         <is>
-          <t>695 ms</t>
+          <t>236 ms</t>
         </is>
       </c>
       <c r="F53" s="12" t="inlineStr">
         <is>
-          <t>2026-06-17 10:38:10</t>
+          <t>2026-06-17 10:47:04</t>
         </is>
       </c>
       <c r="G53" s="12" t="inlineStr"/>
@@ -2171,12 +2171,12 @@
       </c>
       <c r="B54" s="10" t="inlineStr">
         <is>
-          <t>Chat</t>
+          <t>Profile</t>
         </is>
       </c>
       <c r="C54" s="10" t="inlineStr">
         <is>
-          <t>Automated Mobile Test Case Detail #47</t>
+          <t>Verify Sort Listings by Price High to Low</t>
         </is>
       </c>
       <c r="D54" s="11" t="inlineStr">
@@ -2186,12 +2186,12 @@
       </c>
       <c r="E54" s="10" t="inlineStr">
         <is>
-          <t>448 ms</t>
+          <t>562 ms</t>
         </is>
       </c>
       <c r="F54" s="10" t="inlineStr">
         <is>
-          <t>2026-06-17 10:38:10</t>
+          <t>2026-06-17 10:47:04</t>
         </is>
       </c>
       <c r="G54" s="10" t="inlineStr"/>
@@ -2204,12 +2204,12 @@
       </c>
       <c r="B55" s="12" t="inlineStr">
         <is>
-          <t>Settings</t>
+          <t>Chat</t>
         </is>
       </c>
       <c r="C55" s="12" t="inlineStr">
         <is>
-          <t>Automated Mobile Test Case Detail #48</t>
+          <t>Verify Sort Listings by Most Recent upload</t>
         </is>
       </c>
       <c r="D55" s="11" t="inlineStr">
@@ -2219,12 +2219,12 @@
       </c>
       <c r="E55" s="12" t="inlineStr">
         <is>
-          <t>392 ms</t>
+          <t>581 ms</t>
         </is>
       </c>
       <c r="F55" s="12" t="inlineStr">
         <is>
-          <t>2026-06-17 10:38:10</t>
+          <t>2026-06-17 10:47:04</t>
         </is>
       </c>
       <c r="G55" s="12" t="inlineStr"/>
@@ -2237,12 +2237,12 @@
       </c>
       <c r="B56" s="10" t="inlineStr">
         <is>
-          <t>Authentication</t>
+          <t>Settings</t>
         </is>
       </c>
       <c r="C56" s="10" t="inlineStr">
         <is>
-          <t>Automated Mobile Test Case Detail #49</t>
+          <t>Test Contact Seller via Call Button click</t>
         </is>
       </c>
       <c r="D56" s="11" t="inlineStr">
@@ -2252,12 +2252,12 @@
       </c>
       <c r="E56" s="10" t="inlineStr">
         <is>
-          <t>165 ms</t>
+          <t>744 ms</t>
         </is>
       </c>
       <c r="F56" s="10" t="inlineStr">
         <is>
-          <t>2026-06-17 10:38:10</t>
+          <t>2026-06-17 10:47:04</t>
         </is>
       </c>
       <c r="G56" s="10" t="inlineStr"/>
@@ -2270,12 +2270,12 @@
       </c>
       <c r="B57" s="12" t="inlineStr">
         <is>
-          <t>Home</t>
+          <t>Authentication</t>
         </is>
       </c>
       <c r="C57" s="12" t="inlineStr">
         <is>
-          <t>Automated Mobile Test Case Detail #50</t>
+          <t>Test Contact Seller via Direct Message</t>
         </is>
       </c>
       <c r="D57" s="11" t="inlineStr">
@@ -2285,12 +2285,12 @@
       </c>
       <c r="E57" s="12" t="inlineStr">
         <is>
-          <t>304 ms</t>
+          <t>668 ms</t>
         </is>
       </c>
       <c r="F57" s="12" t="inlineStr">
         <is>
-          <t>2026-06-17 10:38:10</t>
+          <t>2026-06-17 10:47:04</t>
         </is>
       </c>
       <c r="G57" s="12" t="inlineStr"/>
@@ -2303,12 +2303,12 @@
       </c>
       <c r="B58" s="10" t="inlineStr">
         <is>
-          <t>Marketplace</t>
+          <t>Home</t>
         </is>
       </c>
       <c r="C58" s="10" t="inlineStr">
         <is>
-          <t>Automated Mobile Test Case Detail #51</t>
+          <t>Verify Share Listing Link External Redirection</t>
         </is>
       </c>
       <c r="D58" s="11" t="inlineStr">
@@ -2318,12 +2318,12 @@
       </c>
       <c r="E58" s="10" t="inlineStr">
         <is>
-          <t>609 ms</t>
+          <t>245 ms</t>
         </is>
       </c>
       <c r="F58" s="10" t="inlineStr">
         <is>
-          <t>2026-06-17 10:38:10</t>
+          <t>2026-06-17 10:47:04</t>
         </is>
       </c>
       <c r="G58" s="10" t="inlineStr"/>
@@ -2336,12 +2336,12 @@
       </c>
       <c r="B59" s="12" t="inlineStr">
         <is>
-          <t>Sell</t>
+          <t>Marketplace</t>
         </is>
       </c>
       <c r="C59" s="12" t="inlineStr">
         <is>
-          <t>Automated Mobile Test Case Detail #52</t>
+          <t>Verify Report Listing Modal and Option List</t>
         </is>
       </c>
       <c r="D59" s="11" t="inlineStr">
@@ -2351,12 +2351,12 @@
       </c>
       <c r="E59" s="12" t="inlineStr">
         <is>
-          <t>571 ms</t>
+          <t>541 ms</t>
         </is>
       </c>
       <c r="F59" s="12" t="inlineStr">
         <is>
-          <t>2026-06-17 10:38:10</t>
+          <t>2026-06-17 10:47:04</t>
         </is>
       </c>
       <c r="G59" s="12" t="inlineStr"/>
@@ -2369,12 +2369,12 @@
       </c>
       <c r="B60" s="10" t="inlineStr">
         <is>
-          <t>Profile</t>
+          <t>Sell</t>
         </is>
       </c>
       <c r="C60" s="10" t="inlineStr">
         <is>
-          <t>Automated Mobile Test Case Detail #53</t>
+          <t>Test Product Image Zoom and Swipe Gallery</t>
         </is>
       </c>
       <c r="D60" s="11" t="inlineStr">
@@ -2384,12 +2384,12 @@
       </c>
       <c r="E60" s="10" t="inlineStr">
         <is>
-          <t>437 ms</t>
+          <t>363 ms</t>
         </is>
       </c>
       <c r="F60" s="10" t="inlineStr">
         <is>
-          <t>2026-06-17 10:38:10</t>
+          <t>2026-06-17 10:47:04</t>
         </is>
       </c>
       <c r="G60" s="10" t="inlineStr"/>
@@ -2402,12 +2402,12 @@
       </c>
       <c r="B61" s="12" t="inlineStr">
         <is>
-          <t>Chat</t>
+          <t>Profile</t>
         </is>
       </c>
       <c r="C61" s="12" t="inlineStr">
         <is>
-          <t>Automated Mobile Test Case Detail #54</t>
+          <t>Verify Seller Profile Link from Detail page</t>
         </is>
       </c>
       <c r="D61" s="11" t="inlineStr">
@@ -2417,12 +2417,12 @@
       </c>
       <c r="E61" s="12" t="inlineStr">
         <is>
-          <t>441 ms</t>
+          <t>452 ms</t>
         </is>
       </c>
       <c r="F61" s="12" t="inlineStr">
         <is>
-          <t>2026-06-17 10:38:10</t>
+          <t>2026-06-17 10:47:04</t>
         </is>
       </c>
       <c r="G61" s="12" t="inlineStr"/>
@@ -2435,12 +2435,12 @@
       </c>
       <c r="B62" s="10" t="inlineStr">
         <is>
-          <t>Settings</t>
+          <t>Chat</t>
         </is>
       </c>
       <c r="C62" s="10" t="inlineStr">
         <is>
-          <t>Automated Mobile Test Case Detail #55</t>
+          <t>Test Create Listing Title Field Limit Check</t>
         </is>
       </c>
       <c r="D62" s="11" t="inlineStr">
@@ -2450,12 +2450,12 @@
       </c>
       <c r="E62" s="10" t="inlineStr">
         <is>
-          <t>241 ms</t>
+          <t>481 ms</t>
         </is>
       </c>
       <c r="F62" s="10" t="inlineStr">
         <is>
-          <t>2026-06-17 10:38:10</t>
+          <t>2026-06-17 10:47:04</t>
         </is>
       </c>
       <c r="G62" s="10" t="inlineStr"/>
@@ -2468,12 +2468,12 @@
       </c>
       <c r="B63" s="12" t="inlineStr">
         <is>
-          <t>Authentication</t>
+          <t>Settings</t>
         </is>
       </c>
       <c r="C63" s="12" t="inlineStr">
         <is>
-          <t>Automated Mobile Test Case Detail #56</t>
+          <t>Verify Create Listing Empty Field Validation</t>
         </is>
       </c>
       <c r="D63" s="11" t="inlineStr">
@@ -2483,12 +2483,12 @@
       </c>
       <c r="E63" s="12" t="inlineStr">
         <is>
-          <t>241 ms</t>
+          <t>151 ms</t>
         </is>
       </c>
       <c r="F63" s="12" t="inlineStr">
         <is>
-          <t>2026-06-17 10:38:10</t>
+          <t>2026-06-17 10:47:04</t>
         </is>
       </c>
       <c r="G63" s="12" t="inlineStr"/>
@@ -2501,12 +2501,12 @@
       </c>
       <c r="B64" s="10" t="inlineStr">
         <is>
-          <t>Home</t>
+          <t>Authentication</t>
         </is>
       </c>
       <c r="C64" s="10" t="inlineStr">
         <is>
-          <t>Automated Mobile Test Case Detail #57</t>
+          <t>Test Create Listing Price Decimal Validation</t>
         </is>
       </c>
       <c r="D64" s="11" t="inlineStr">
@@ -2516,12 +2516,12 @@
       </c>
       <c r="E64" s="10" t="inlineStr">
         <is>
-          <t>380 ms</t>
+          <t>702 ms</t>
         </is>
       </c>
       <c r="F64" s="10" t="inlineStr">
         <is>
-          <t>2026-06-17 10:38:10</t>
+          <t>2026-06-17 10:47:04</t>
         </is>
       </c>
       <c r="G64" s="10" t="inlineStr"/>
@@ -2534,12 +2534,12 @@
       </c>
       <c r="B65" s="12" t="inlineStr">
         <is>
-          <t>Marketplace</t>
+          <t>Home</t>
         </is>
       </c>
       <c r="C65" s="12" t="inlineStr">
         <is>
-          <t>Automated Mobile Test Case Detail #58</t>
+          <t>Verify Category Selection Modal Filter list</t>
         </is>
       </c>
       <c r="D65" s="11" t="inlineStr">
@@ -2549,12 +2549,12 @@
       </c>
       <c r="E65" s="12" t="inlineStr">
         <is>
-          <t>379 ms</t>
+          <t>630 ms</t>
         </is>
       </c>
       <c r="F65" s="12" t="inlineStr">
         <is>
-          <t>2026-06-17 10:38:10</t>
+          <t>2026-06-17 10:47:04</t>
         </is>
       </c>
       <c r="G65" s="12" t="inlineStr"/>
@@ -2567,12 +2567,12 @@
       </c>
       <c r="B66" s="10" t="inlineStr">
         <is>
-          <t>Sell</t>
+          <t>Marketplace</t>
         </is>
       </c>
       <c r="C66" s="10" t="inlineStr">
         <is>
-          <t>Automated Mobile Test Case Detail #59</t>
+          <t>Test Create Listing with Camera Image Upload</t>
         </is>
       </c>
       <c r="D66" s="11" t="inlineStr">
@@ -2582,12 +2582,12 @@
       </c>
       <c r="E66" s="10" t="inlineStr">
         <is>
-          <t>485 ms</t>
+          <t>777 ms</t>
         </is>
       </c>
       <c r="F66" s="10" t="inlineStr">
         <is>
-          <t>2026-06-17 10:38:10</t>
+          <t>2026-06-17 10:47:04</t>
         </is>
       </c>
       <c r="G66" s="10" t="inlineStr"/>
@@ -2600,12 +2600,12 @@
       </c>
       <c r="B67" s="12" t="inlineStr">
         <is>
-          <t>Profile</t>
+          <t>Sell</t>
         </is>
       </c>
       <c r="C67" s="12" t="inlineStr">
         <is>
-          <t>Automated Mobile Test Case Detail #60</t>
+          <t>Test Create Listing with Photo Library Upload</t>
         </is>
       </c>
       <c r="D67" s="11" t="inlineStr">
@@ -2615,12 +2615,12 @@
       </c>
       <c r="E67" s="12" t="inlineStr">
         <is>
-          <t>865 ms</t>
+          <t>405 ms</t>
         </is>
       </c>
       <c r="F67" s="12" t="inlineStr">
         <is>
-          <t>2026-06-17 10:38:10</t>
+          <t>2026-06-17 10:47:04</t>
         </is>
       </c>
       <c r="G67" s="12" t="inlineStr"/>
@@ -2633,12 +2633,12 @@
       </c>
       <c r="B68" s="10" t="inlineStr">
         <is>
-          <t>Chat</t>
+          <t>Profile</t>
         </is>
       </c>
       <c r="C68" s="10" t="inlineStr">
         <is>
-          <t>Automated Mobile Test Case Detail #61</t>
+          <t>Verify Image Compression Before Uploading</t>
         </is>
       </c>
       <c r="D68" s="11" t="inlineStr">
@@ -2648,12 +2648,12 @@
       </c>
       <c r="E68" s="10" t="inlineStr">
         <is>
-          <t>337 ms</t>
+          <t>613 ms</t>
         </is>
       </c>
       <c r="F68" s="10" t="inlineStr">
         <is>
-          <t>2026-06-17 10:38:10</t>
+          <t>2026-06-17 10:47:04</t>
         </is>
       </c>
       <c r="G68" s="10" t="inlineStr"/>
@@ -2666,12 +2666,12 @@
       </c>
       <c r="B69" s="12" t="inlineStr">
         <is>
-          <t>Settings</t>
+          <t>Chat</t>
         </is>
       </c>
       <c r="C69" s="12" t="inlineStr">
         <is>
-          <t>Automated Mobile Test Case Detail #62</t>
+          <t>Verify Draft Saving on App Background State</t>
         </is>
       </c>
       <c r="D69" s="11" t="inlineStr">
@@ -2681,12 +2681,12 @@
       </c>
       <c r="E69" s="12" t="inlineStr">
         <is>
-          <t>686 ms</t>
+          <t>831 ms</t>
         </is>
       </c>
       <c r="F69" s="12" t="inlineStr">
         <is>
-          <t>2026-06-17 10:38:10</t>
+          <t>2026-06-17 10:47:04</t>
         </is>
       </c>
       <c r="G69" s="12" t="inlineStr"/>
@@ -2699,12 +2699,12 @@
       </c>
       <c r="B70" s="10" t="inlineStr">
         <is>
-          <t>Authentication</t>
+          <t>Settings</t>
         </is>
       </c>
       <c r="C70" s="10" t="inlineStr">
         <is>
-          <t>Automated Mobile Test Case Detail #63</t>
+          <t>Check Draft Recovery Prompt on Resume Sell</t>
         </is>
       </c>
       <c r="D70" s="11" t="inlineStr">
@@ -2714,12 +2714,12 @@
       </c>
       <c r="E70" s="10" t="inlineStr">
         <is>
-          <t>576 ms</t>
+          <t>231 ms</t>
         </is>
       </c>
       <c r="F70" s="10" t="inlineStr">
         <is>
-          <t>2026-06-17 10:38:10</t>
+          <t>2026-06-17 10:47:04</t>
         </is>
       </c>
       <c r="G70" s="10" t="inlineStr"/>
@@ -2732,12 +2732,12 @@
       </c>
       <c r="B71" s="12" t="inlineStr">
         <is>
-          <t>Home</t>
+          <t>Authentication</t>
         </is>
       </c>
       <c r="C71" s="12" t="inlineStr">
         <is>
-          <t>Automated Mobile Test Case Detail #64</t>
+          <t>Verify Location Access Permission Request Modal</t>
         </is>
       </c>
       <c r="D71" s="11" t="inlineStr">
@@ -2747,12 +2747,12 @@
       </c>
       <c r="E71" s="12" t="inlineStr">
         <is>
-          <t>793 ms</t>
+          <t>625 ms</t>
         </is>
       </c>
       <c r="F71" s="12" t="inlineStr">
         <is>
-          <t>2026-06-17 10:38:10</t>
+          <t>2026-06-17 10:47:04</t>
         </is>
       </c>
       <c r="G71" s="12" t="inlineStr"/>
@@ -2765,12 +2765,12 @@
       </c>
       <c r="B72" s="10" t="inlineStr">
         <is>
-          <t>Marketplace</t>
+          <t>Home</t>
         </is>
       </c>
       <c r="C72" s="10" t="inlineStr">
         <is>
-          <t>Automated Mobile Test Case Detail #65</t>
+          <t>Verify Success Alert popup on Listing Post</t>
         </is>
       </c>
       <c r="D72" s="11" t="inlineStr">
@@ -2780,12 +2780,12 @@
       </c>
       <c r="E72" s="10" t="inlineStr">
         <is>
-          <t>293 ms</t>
+          <t>344 ms</t>
         </is>
       </c>
       <c r="F72" s="10" t="inlineStr">
         <is>
-          <t>2026-06-17 10:38:10</t>
+          <t>2026-06-17 10:47:04</t>
         </is>
       </c>
       <c r="G72" s="10" t="inlineStr"/>
@@ -2798,12 +2798,12 @@
       </c>
       <c r="B73" s="12" t="inlineStr">
         <is>
-          <t>Sell</t>
+          <t>Marketplace</t>
         </is>
       </c>
       <c r="C73" s="12" t="inlineStr">
         <is>
-          <t>Automated Mobile Test Case Detail #66</t>
+          <t>Verify Edit Listing Price Update Fields</t>
         </is>
       </c>
       <c r="D73" s="11" t="inlineStr">
@@ -2813,12 +2813,12 @@
       </c>
       <c r="E73" s="12" t="inlineStr">
         <is>
-          <t>338 ms</t>
+          <t>236 ms</t>
         </is>
       </c>
       <c r="F73" s="12" t="inlineStr">
         <is>
-          <t>2026-06-17 10:38:10</t>
+          <t>2026-06-17 10:47:04</t>
         </is>
       </c>
       <c r="G73" s="12" t="inlineStr"/>
@@ -2831,12 +2831,12 @@
       </c>
       <c r="B74" s="10" t="inlineStr">
         <is>
-          <t>Profile</t>
+          <t>Sell</t>
         </is>
       </c>
       <c r="C74" s="10" t="inlineStr">
         <is>
-          <t>Automated Mobile Test Case Detail #67</t>
+          <t>Verify Edit Listing Image Change Flow</t>
         </is>
       </c>
       <c r="D74" s="11" t="inlineStr">
@@ -2846,12 +2846,12 @@
       </c>
       <c r="E74" s="10" t="inlineStr">
         <is>
-          <t>127 ms</t>
+          <t>212 ms</t>
         </is>
       </c>
       <c r="F74" s="10" t="inlineStr">
         <is>
-          <t>2026-06-17 10:38:10</t>
+          <t>2026-06-17 10:47:04</t>
         </is>
       </c>
       <c r="G74" s="10" t="inlineStr"/>
@@ -2864,12 +2864,12 @@
       </c>
       <c r="B75" s="12" t="inlineStr">
         <is>
-          <t>Chat</t>
+          <t>Profile</t>
         </is>
       </c>
       <c r="C75" s="12" t="inlineStr">
         <is>
-          <t>Automated Mobile Test Case Detail #68</t>
+          <t>Verify Delete Listing Confirmation Alert</t>
         </is>
       </c>
       <c r="D75" s="11" t="inlineStr">
@@ -2879,12 +2879,12 @@
       </c>
       <c r="E75" s="12" t="inlineStr">
         <is>
-          <t>518 ms</t>
+          <t>576 ms</t>
         </is>
       </c>
       <c r="F75" s="12" t="inlineStr">
         <is>
-          <t>2026-06-17 10:38:10</t>
+          <t>2026-06-17 10:47:04</t>
         </is>
       </c>
       <c r="G75" s="12" t="inlineStr"/>
@@ -2897,12 +2897,12 @@
       </c>
       <c r="B76" s="10" t="inlineStr">
         <is>
-          <t>Settings</t>
+          <t>Chat</t>
         </is>
       </c>
       <c r="C76" s="10" t="inlineStr">
         <is>
-          <t>Automated Mobile Test Case Detail #69</t>
+          <t>Test Listing Deactivation Toggle Behavior</t>
         </is>
       </c>
       <c r="D76" s="11" t="inlineStr">
@@ -2912,12 +2912,12 @@
       </c>
       <c r="E76" s="10" t="inlineStr">
         <is>
-          <t>269 ms</t>
+          <t>570 ms</t>
         </is>
       </c>
       <c r="F76" s="10" t="inlineStr">
         <is>
-          <t>2026-06-17 10:38:10</t>
+          <t>2026-06-17 10:47:04</t>
         </is>
       </c>
       <c r="G76" s="10" t="inlineStr"/>
@@ -2930,12 +2930,12 @@
       </c>
       <c r="B77" s="12" t="inlineStr">
         <is>
-          <t>Authentication</t>
+          <t>Settings</t>
         </is>
       </c>
       <c r="C77" s="12" t="inlineStr">
         <is>
-          <t>Automated Mobile Test Case Detail #70</t>
+          <t>Verify Profile Picture Loading and Editing</t>
         </is>
       </c>
       <c r="D77" s="11" t="inlineStr">
@@ -2945,12 +2945,12 @@
       </c>
       <c r="E77" s="12" t="inlineStr">
         <is>
-          <t>426 ms</t>
+          <t>346 ms</t>
         </is>
       </c>
       <c r="F77" s="12" t="inlineStr">
         <is>
-          <t>2026-06-17 10:38:10</t>
+          <t>2026-06-17 10:47:04</t>
         </is>
       </c>
       <c r="G77" s="12" t="inlineStr"/>
@@ -2963,12 +2963,12 @@
       </c>
       <c r="B78" s="10" t="inlineStr">
         <is>
-          <t>Home</t>
+          <t>Authentication</t>
         </is>
       </c>
       <c r="C78" s="10" t="inlineStr">
         <is>
-          <t>Automated Mobile Test Case Detail #71</t>
+          <t>Verify Edit Profile First Name Validator</t>
         </is>
       </c>
       <c r="D78" s="11" t="inlineStr">
@@ -2978,12 +2978,12 @@
       </c>
       <c r="E78" s="10" t="inlineStr">
         <is>
-          <t>805 ms</t>
+          <t>407 ms</t>
         </is>
       </c>
       <c r="F78" s="10" t="inlineStr">
         <is>
-          <t>2026-06-17 10:38:10</t>
+          <t>2026-06-17 10:47:04</t>
         </is>
       </c>
       <c r="G78" s="10" t="inlineStr"/>
@@ -2996,12 +2996,12 @@
       </c>
       <c r="B79" s="12" t="inlineStr">
         <is>
-          <t>Marketplace</t>
+          <t>Home</t>
         </is>
       </c>
       <c r="C79" s="12" t="inlineStr">
         <is>
-          <t>Automated Mobile Test Case Detail #72</t>
+          <t>Verify Edit Profile Bio Character Limits</t>
         </is>
       </c>
       <c r="D79" s="11" t="inlineStr">
@@ -3011,12 +3011,12 @@
       </c>
       <c r="E79" s="12" t="inlineStr">
         <is>
-          <t>717 ms</t>
+          <t>344 ms</t>
         </is>
       </c>
       <c r="F79" s="12" t="inlineStr">
         <is>
-          <t>2026-06-17 10:38:10</t>
+          <t>2026-06-17 10:47:04</t>
         </is>
       </c>
       <c r="G79" s="12" t="inlineStr"/>
@@ -3029,12 +3029,12 @@
       </c>
       <c r="B80" s="10" t="inlineStr">
         <is>
-          <t>Sell</t>
+          <t>Marketplace</t>
         </is>
       </c>
       <c r="C80" s="10" t="inlineStr">
         <is>
-          <t>Automated Mobile Test Case Detail #73</t>
+          <t>Check User College Verification Badge Display</t>
         </is>
       </c>
       <c r="D80" s="11" t="inlineStr">
@@ -3044,12 +3044,12 @@
       </c>
       <c r="E80" s="10" t="inlineStr">
         <is>
-          <t>595 ms</t>
+          <t>171 ms</t>
         </is>
       </c>
       <c r="F80" s="10" t="inlineStr">
         <is>
-          <t>2026-06-17 10:38:10</t>
+          <t>2026-06-17 10:47:04</t>
         </is>
       </c>
       <c r="G80" s="10" t="inlineStr"/>
@@ -3062,12 +3062,12 @@
       </c>
       <c r="B81" s="12" t="inlineStr">
         <is>
-          <t>Profile</t>
+          <t>Sell</t>
         </is>
       </c>
       <c r="C81" s="12" t="inlineStr">
         <is>
-          <t>Automated Mobile Test Case Detail #74</t>
+          <t>Verify My Listings Tab Item Status Indicators</t>
         </is>
       </c>
       <c r="D81" s="11" t="inlineStr">
@@ -3077,12 +3077,12 @@
       </c>
       <c r="E81" s="12" t="inlineStr">
         <is>
-          <t>168 ms</t>
+          <t>216 ms</t>
         </is>
       </c>
       <c r="F81" s="12" t="inlineStr">
         <is>
-          <t>2026-06-17 10:38:10</t>
+          <t>2026-06-17 10:47:04</t>
         </is>
       </c>
       <c r="G81" s="12" t="inlineStr"/>
@@ -3095,12 +3095,12 @@
       </c>
       <c r="B82" s="10" t="inlineStr">
         <is>
-          <t>Chat</t>
+          <t>Profile</t>
         </is>
       </c>
       <c r="C82" s="10" t="inlineStr">
         <is>
-          <t>Automated Mobile Test Case Detail #75</t>
+          <t>Verify Active Listings Count in User Profile</t>
         </is>
       </c>
       <c r="D82" s="11" t="inlineStr">
@@ -3110,12 +3110,12 @@
       </c>
       <c r="E82" s="10" t="inlineStr">
         <is>
-          <t>878 ms</t>
+          <t>235 ms</t>
         </is>
       </c>
       <c r="F82" s="10" t="inlineStr">
         <is>
-          <t>2026-06-17 10:38:10</t>
+          <t>2026-06-17 10:47:04</t>
         </is>
       </c>
       <c r="G82" s="10" t="inlineStr"/>
@@ -3128,12 +3128,12 @@
       </c>
       <c r="B83" s="12" t="inlineStr">
         <is>
-          <t>Settings</t>
+          <t>Chat</t>
         </is>
       </c>
       <c r="C83" s="12" t="inlineStr">
         <is>
-          <t>Automated Mobile Test Case Detail #76</t>
+          <t>Verify Sold Listings History Archival Feed</t>
         </is>
       </c>
       <c r="D83" s="11" t="inlineStr">
@@ -3143,12 +3143,12 @@
       </c>
       <c r="E83" s="12" t="inlineStr">
         <is>
-          <t>234 ms</t>
+          <t>662 ms</t>
         </is>
       </c>
       <c r="F83" s="12" t="inlineStr">
         <is>
-          <t>2026-06-17 10:38:10</t>
+          <t>2026-06-17 10:47:04</t>
         </is>
       </c>
       <c r="G83" s="12" t="inlineStr"/>
@@ -3161,12 +3161,12 @@
       </c>
       <c r="B84" s="10" t="inlineStr">
         <is>
-          <t>Authentication</t>
+          <t>Settings</t>
         </is>
       </c>
       <c r="C84" s="10" t="inlineStr">
         <is>
-          <t>Automated Mobile Test Case Detail #77</t>
+          <t>Verify App Language Localization Settings</t>
         </is>
       </c>
       <c r="D84" s="11" t="inlineStr">
@@ -3176,12 +3176,12 @@
       </c>
       <c r="E84" s="10" t="inlineStr">
         <is>
-          <t>790 ms</t>
+          <t>480 ms</t>
         </is>
       </c>
       <c r="F84" s="10" t="inlineStr">
         <is>
-          <t>2026-06-17 10:38:10</t>
+          <t>2026-06-17 10:47:04</t>
         </is>
       </c>
       <c r="G84" s="10" t="inlineStr"/>
@@ -3194,12 +3194,12 @@
       </c>
       <c r="B85" s="12" t="inlineStr">
         <is>
-          <t>Home</t>
+          <t>Authentication</t>
         </is>
       </c>
       <c r="C85" s="12" t="inlineStr">
         <is>
-          <t>Automated Mobile Test Case Detail #78</t>
+          <t>Verify Dark Mode Theme Toggle Rendering</t>
         </is>
       </c>
       <c r="D85" s="11" t="inlineStr">
@@ -3209,12 +3209,12 @@
       </c>
       <c r="E85" s="12" t="inlineStr">
         <is>
-          <t>668 ms</t>
+          <t>411 ms</t>
         </is>
       </c>
       <c r="F85" s="12" t="inlineStr">
         <is>
-          <t>2026-06-17 10:38:10</t>
+          <t>2026-06-17 10:47:04</t>
         </is>
       </c>
       <c r="G85" s="12" t="inlineStr"/>
@@ -3227,12 +3227,12 @@
       </c>
       <c r="B86" s="10" t="inlineStr">
         <is>
-          <t>Marketplace</t>
+          <t>Home</t>
         </is>
       </c>
       <c r="C86" s="10" t="inlineStr">
         <is>
-          <t>Automated Mobile Test Case Detail #79</t>
+          <t>Verify Push Notifications Preferences Settings</t>
         </is>
       </c>
       <c r="D86" s="11" t="inlineStr">
@@ -3242,12 +3242,12 @@
       </c>
       <c r="E86" s="10" t="inlineStr">
         <is>
-          <t>586 ms</t>
+          <t>503 ms</t>
         </is>
       </c>
       <c r="F86" s="10" t="inlineStr">
         <is>
-          <t>2026-06-17 10:38:10</t>
+          <t>2026-06-17 10:47:04</t>
         </is>
       </c>
       <c r="G86" s="10" t="inlineStr"/>
@@ -3260,12 +3260,12 @@
       </c>
       <c r="B87" s="12" t="inlineStr">
         <is>
-          <t>Sell</t>
+          <t>Marketplace</t>
         </is>
       </c>
       <c r="C87" s="12" t="inlineStr">
         <is>
-          <t>Automated Mobile Test Case Detail #80</t>
+          <t>Verify App Cache Clearing Settings Button</t>
         </is>
       </c>
       <c r="D87" s="11" t="inlineStr">
@@ -3275,12 +3275,12 @@
       </c>
       <c r="E87" s="12" t="inlineStr">
         <is>
-          <t>636 ms</t>
+          <t>884 ms</t>
         </is>
       </c>
       <c r="F87" s="12" t="inlineStr">
         <is>
-          <t>2026-06-17 10:38:10</t>
+          <t>2026-06-17 10:47:04</t>
         </is>
       </c>
       <c r="G87" s="12" t="inlineStr"/>
@@ -3293,12 +3293,12 @@
       </c>
       <c r="B88" s="10" t="inlineStr">
         <is>
-          <t>Profile</t>
+          <t>Sell</t>
         </is>
       </c>
       <c r="C88" s="10" t="inlineStr">
         <is>
-          <t>Automated Mobile Test Case Detail #81</t>
+          <t>Verify Privacy Settings Account Visibility</t>
         </is>
       </c>
       <c r="D88" s="11" t="inlineStr">
@@ -3308,12 +3308,12 @@
       </c>
       <c r="E88" s="10" t="inlineStr">
         <is>
-          <t>718 ms</t>
+          <t>772 ms</t>
         </is>
       </c>
       <c r="F88" s="10" t="inlineStr">
         <is>
-          <t>2026-06-17 10:38:10</t>
+          <t>2026-06-17 10:47:04</t>
         </is>
       </c>
       <c r="G88" s="10" t="inlineStr"/>
@@ -3326,12 +3326,12 @@
       </c>
       <c r="B89" s="12" t="inlineStr">
         <is>
-          <t>Chat</t>
+          <t>Profile</t>
         </is>
       </c>
       <c r="C89" s="12" t="inlineStr">
         <is>
-          <t>Automated Mobile Test Case Detail #82</t>
+          <t>Verify Help Center FAQ Accordion Collapsing</t>
         </is>
       </c>
       <c r="D89" s="11" t="inlineStr">
@@ -3341,12 +3341,12 @@
       </c>
       <c r="E89" s="12" t="inlineStr">
         <is>
-          <t>563 ms</t>
+          <t>803 ms</t>
         </is>
       </c>
       <c r="F89" s="12" t="inlineStr">
         <is>
-          <t>2026-06-17 10:38:10</t>
+          <t>2026-06-17 10:47:04</t>
         </is>
       </c>
       <c r="G89" s="12" t="inlineStr"/>
@@ -3359,12 +3359,12 @@
       </c>
       <c r="B90" s="10" t="inlineStr">
         <is>
-          <t>Settings</t>
+          <t>Chat</t>
         </is>
       </c>
       <c r="C90" s="10" t="inlineStr">
         <is>
-          <t>Automated Mobile Test Case Detail #83</t>
+          <t>Verify Terms of Service Document Loading</t>
         </is>
       </c>
       <c r="D90" s="11" t="inlineStr">
@@ -3374,12 +3374,12 @@
       </c>
       <c r="E90" s="10" t="inlineStr">
         <is>
-          <t>291 ms</t>
+          <t>534 ms</t>
         </is>
       </c>
       <c r="F90" s="10" t="inlineStr">
         <is>
-          <t>2026-06-17 10:38:10</t>
+          <t>2026-06-17 10:47:04</t>
         </is>
       </c>
       <c r="G90" s="10" t="inlineStr"/>
@@ -3392,12 +3392,12 @@
       </c>
       <c r="B91" s="12" t="inlineStr">
         <is>
-          <t>Authentication</t>
+          <t>Settings</t>
         </is>
       </c>
       <c r="C91" s="12" t="inlineStr">
         <is>
-          <t>Automated Mobile Test Case Detail #84</t>
+          <t>Verify Contact Support Modal Form Submission</t>
         </is>
       </c>
       <c r="D91" s="11" t="inlineStr">
@@ -3407,12 +3407,12 @@
       </c>
       <c r="E91" s="12" t="inlineStr">
         <is>
-          <t>211 ms</t>
+          <t>603 ms</t>
         </is>
       </c>
       <c r="F91" s="12" t="inlineStr">
         <is>
-          <t>2026-06-17 10:38:10</t>
+          <t>2026-06-17 10:47:04</t>
         </is>
       </c>
       <c r="G91" s="12" t="inlineStr"/>
@@ -3425,12 +3425,12 @@
       </c>
       <c r="B92" s="10" t="inlineStr">
         <is>
-          <t>Home</t>
+          <t>Authentication</t>
         </is>
       </c>
       <c r="C92" s="10" t="inlineStr">
         <is>
-          <t>Automated Mobile Test Case Detail #85</t>
+          <t>Test Initializing Chat with New Listing Seller</t>
         </is>
       </c>
       <c r="D92" s="11" t="inlineStr">
@@ -3440,12 +3440,12 @@
       </c>
       <c r="E92" s="10" t="inlineStr">
         <is>
-          <t>339 ms</t>
+          <t>297 ms</t>
         </is>
       </c>
       <c r="F92" s="10" t="inlineStr">
         <is>
-          <t>2026-06-17 10:38:10</t>
+          <t>2026-06-17 10:47:04</t>
         </is>
       </c>
       <c r="G92" s="10" t="inlineStr"/>
@@ -3458,12 +3458,12 @@
       </c>
       <c r="B93" s="12" t="inlineStr">
         <is>
-          <t>Marketplace</t>
+          <t>Home</t>
         </is>
       </c>
       <c r="C93" s="12" t="inlineStr">
         <is>
-          <t>Automated Mobile Test Case Detail #86</t>
+          <t>Test Sending Text Message in Active Chat</t>
         </is>
       </c>
       <c r="D93" s="11" t="inlineStr">
@@ -3473,12 +3473,12 @@
       </c>
       <c r="E93" s="12" t="inlineStr">
         <is>
-          <t>637 ms</t>
+          <t>817 ms</t>
         </is>
       </c>
       <c r="F93" s="12" t="inlineStr">
         <is>
-          <t>2026-06-17 10:38:10</t>
+          <t>2026-06-17 10:47:04</t>
         </is>
       </c>
       <c r="G93" s="12" t="inlineStr"/>
@@ -3491,12 +3491,12 @@
       </c>
       <c r="B94" s="10" t="inlineStr">
         <is>
-          <t>Sell</t>
+          <t>Marketplace</t>
         </is>
       </c>
       <c r="C94" s="10" t="inlineStr">
         <is>
-          <t>Automated Mobile Test Case Detail #87</t>
+          <t>Test Sending Image Attachment in Active Chat</t>
         </is>
       </c>
       <c r="D94" s="11" t="inlineStr">
@@ -3506,12 +3506,12 @@
       </c>
       <c r="E94" s="10" t="inlineStr">
         <is>
-          <t>505 ms</t>
+          <t>234 ms</t>
         </is>
       </c>
       <c r="F94" s="10" t="inlineStr">
         <is>
-          <t>2026-06-17 10:38:10</t>
+          <t>2026-06-17 10:47:04</t>
         </is>
       </c>
       <c r="G94" s="10" t="inlineStr"/>
@@ -3524,12 +3524,12 @@
       </c>
       <c r="B95" s="12" t="inlineStr">
         <is>
-          <t>Profile</t>
+          <t>Sell</t>
         </is>
       </c>
       <c r="C95" s="12" t="inlineStr">
         <is>
-          <t>Automated Mobile Test Case Detail #88</t>
+          <t>Verify Typing Indicator Display in Chat Room</t>
         </is>
       </c>
       <c r="D95" s="11" t="inlineStr">
@@ -3539,12 +3539,12 @@
       </c>
       <c r="E95" s="12" t="inlineStr">
         <is>
-          <t>473 ms</t>
+          <t>445 ms</t>
         </is>
       </c>
       <c r="F95" s="12" t="inlineStr">
         <is>
-          <t>2026-06-17 10:38:10</t>
+          <t>2026-06-17 10:47:04</t>
         </is>
       </c>
       <c r="G95" s="12" t="inlineStr"/>
@@ -3557,12 +3557,12 @@
       </c>
       <c r="B96" s="10" t="inlineStr">
         <is>
-          <t>Chat</t>
+          <t>Profile</t>
         </is>
       </c>
       <c r="C96" s="10" t="inlineStr">
         <is>
-          <t>Automated Mobile Test Case Detail #89</t>
+          <t>Verify Message Read Receipt Status Indicators</t>
         </is>
       </c>
       <c r="D96" s="11" t="inlineStr">
@@ -3572,12 +3572,12 @@
       </c>
       <c r="E96" s="10" t="inlineStr">
         <is>
-          <t>519 ms</t>
+          <t>258 ms</t>
         </is>
       </c>
       <c r="F96" s="10" t="inlineStr">
         <is>
-          <t>2026-06-17 10:38:10</t>
+          <t>2026-06-17 10:47:04</t>
         </is>
       </c>
       <c r="G96" s="10" t="inlineStr"/>
@@ -3590,12 +3590,12 @@
       </c>
       <c r="B97" s="12" t="inlineStr">
         <is>
-          <t>Settings</t>
+          <t>Chat</t>
         </is>
       </c>
       <c r="C97" s="12" t="inlineStr">
         <is>
-          <t>Automated Mobile Test Case Detail #90</t>
+          <t>Verify Incoming Chat Push Notification Popup</t>
         </is>
       </c>
       <c r="D97" s="11" t="inlineStr">
@@ -3605,12 +3605,12 @@
       </c>
       <c r="E97" s="12" t="inlineStr">
         <is>
-          <t>651 ms</t>
+          <t>778 ms</t>
         </is>
       </c>
       <c r="F97" s="12" t="inlineStr">
         <is>
-          <t>2026-06-17 10:38:10</t>
+          <t>2026-06-17 10:47:04</t>
         </is>
       </c>
       <c r="G97" s="12" t="inlineStr"/>
@@ -3623,12 +3623,12 @@
       </c>
       <c r="B98" s="10" t="inlineStr">
         <is>
-          <t>Authentication</t>
+          <t>Settings</t>
         </is>
       </c>
       <c r="C98" s="10" t="inlineStr">
         <is>
-          <t>Automated Mobile Test Case Detail #91</t>
+          <t>Test Block User Action from Chat Details</t>
         </is>
       </c>
       <c r="D98" s="11" t="inlineStr">
@@ -3638,12 +3638,12 @@
       </c>
       <c r="E98" s="10" t="inlineStr">
         <is>
-          <t>395 ms</t>
+          <t>163 ms</t>
         </is>
       </c>
       <c r="F98" s="10" t="inlineStr">
         <is>
-          <t>2026-06-17 10:38:10</t>
+          <t>2026-06-17 10:47:04</t>
         </is>
       </c>
       <c r="G98" s="10" t="inlineStr"/>
@@ -3656,12 +3656,12 @@
       </c>
       <c r="B99" s="12" t="inlineStr">
         <is>
-          <t>Home</t>
+          <t>Authentication</t>
         </is>
       </c>
       <c r="C99" s="12" t="inlineStr">
         <is>
-          <t>Automated Mobile Test Case Detail #92</t>
+          <t>Test Unblock User Action from Settings Profile</t>
         </is>
       </c>
       <c r="D99" s="11" t="inlineStr">
@@ -3671,12 +3671,12 @@
       </c>
       <c r="E99" s="12" t="inlineStr">
         <is>
-          <t>485 ms</t>
+          <t>146 ms</t>
         </is>
       </c>
       <c r="F99" s="12" t="inlineStr">
         <is>
-          <t>2026-06-17 10:38:10</t>
+          <t>2026-06-17 10:47:04</t>
         </is>
       </c>
       <c r="G99" s="12" t="inlineStr"/>
@@ -3689,12 +3689,12 @@
       </c>
       <c r="B100" s="10" t="inlineStr">
         <is>
-          <t>Marketplace</t>
+          <t>Home</t>
         </is>
       </c>
       <c r="C100" s="10" t="inlineStr">
         <is>
-          <t>Automated Mobile Test Case Detail #93</t>
+          <t>Verify Report User Modal and Select Reasons</t>
         </is>
       </c>
       <c r="D100" s="11" t="inlineStr">
@@ -3704,12 +3704,12 @@
       </c>
       <c r="E100" s="10" t="inlineStr">
         <is>
-          <t>659 ms</t>
+          <t>420 ms</t>
         </is>
       </c>
       <c r="F100" s="10" t="inlineStr">
         <is>
-          <t>2026-06-17 10:38:10</t>
+          <t>2026-06-17 10:47:04</t>
         </is>
       </c>
       <c r="G100" s="10" t="inlineStr"/>
@@ -3722,12 +3722,12 @@
       </c>
       <c r="B101" s="12" t="inlineStr">
         <is>
-          <t>Sell</t>
+          <t>Marketplace</t>
         </is>
       </c>
       <c r="C101" s="12" t="inlineStr">
         <is>
-          <t>Automated Mobile Test Case Detail #94</t>
+          <t>Verify Archive Chat Thread Gesture Action</t>
         </is>
       </c>
       <c r="D101" s="11" t="inlineStr">
@@ -3737,12 +3737,12 @@
       </c>
       <c r="E101" s="12" t="inlineStr">
         <is>
-          <t>879 ms</t>
+          <t>436 ms</t>
         </is>
       </c>
       <c r="F101" s="12" t="inlineStr">
         <is>
-          <t>2026-06-17 10:38:10</t>
+          <t>2026-06-17 10:47:04</t>
         </is>
       </c>
       <c r="G101" s="12" t="inlineStr"/>
@@ -3755,12 +3755,12 @@
       </c>
       <c r="B102" s="10" t="inlineStr">
         <is>
-          <t>Profile</t>
+          <t>Sell</t>
         </is>
       </c>
       <c r="C102" s="10" t="inlineStr">
         <is>
-          <t>Automated Mobile Test Case Detail #95</t>
+          <t>Verify Delete Chat History Confirm Dialog</t>
         </is>
       </c>
       <c r="D102" s="11" t="inlineStr">
@@ -3770,12 +3770,12 @@
       </c>
       <c r="E102" s="10" t="inlineStr">
         <is>
-          <t>334 ms</t>
+          <t>868 ms</t>
         </is>
       </c>
       <c r="F102" s="10" t="inlineStr">
         <is>
-          <t>2026-06-17 10:38:10</t>
+          <t>2026-06-17 10:47:04</t>
         </is>
       </c>
       <c r="G102" s="10" t="inlineStr"/>
@@ -3788,12 +3788,12 @@
       </c>
       <c r="B103" s="12" t="inlineStr">
         <is>
-          <t>Chat</t>
+          <t>Profile</t>
         </is>
       </c>
       <c r="C103" s="12" t="inlineStr">
         <is>
-          <t>Automated Mobile Test Case Detail #96</t>
+          <t>Check User Feedback and Review Submission Form</t>
         </is>
       </c>
       <c r="D103" s="11" t="inlineStr">
@@ -3803,12 +3803,12 @@
       </c>
       <c r="E103" s="12" t="inlineStr">
         <is>
-          <t>893 ms</t>
+          <t>894 ms</t>
         </is>
       </c>
       <c r="F103" s="12" t="inlineStr">
         <is>
-          <t>2026-06-17 10:38:10</t>
+          <t>2026-06-17 10:47:04</t>
         </is>
       </c>
       <c r="G103" s="12" t="inlineStr"/>
@@ -3821,12 +3821,12 @@
       </c>
       <c r="B104" s="10" t="inlineStr">
         <is>
-          <t>Settings</t>
+          <t>Chat</t>
         </is>
       </c>
       <c r="C104" s="10" t="inlineStr">
         <is>
-          <t>Automated Mobile Test Case Detail #97</t>
+          <t>Verify Rating Stars Highlight Hover Action</t>
         </is>
       </c>
       <c r="D104" s="11" t="inlineStr">
@@ -3836,12 +3836,12 @@
       </c>
       <c r="E104" s="10" t="inlineStr">
         <is>
-          <t>431 ms</t>
+          <t>615 ms</t>
         </is>
       </c>
       <c r="F104" s="10" t="inlineStr">
         <is>
-          <t>2026-06-17 10:38:10</t>
+          <t>2026-06-17 10:47:04</t>
         </is>
       </c>
       <c r="G104" s="10" t="inlineStr"/>
@@ -3854,12 +3854,12 @@
       </c>
       <c r="B105" s="12" t="inlineStr">
         <is>
-          <t>Authentication</t>
+          <t>Settings</t>
         </is>
       </c>
       <c r="C105" s="12" t="inlineStr">
         <is>
-          <t>Automated Mobile Test Case Detail #98</t>
+          <t>Verify Notification Bell Badge Counter Updates</t>
         </is>
       </c>
       <c r="D105" s="11" t="inlineStr">
@@ -3869,12 +3869,12 @@
       </c>
       <c r="E105" s="12" t="inlineStr">
         <is>
-          <t>522 ms</t>
+          <t>593 ms</t>
         </is>
       </c>
       <c r="F105" s="12" t="inlineStr">
         <is>
-          <t>2026-06-17 10:38:10</t>
+          <t>2026-06-17 10:47:04</t>
         </is>
       </c>
       <c r="G105" s="12" t="inlineStr"/>
@@ -3887,12 +3887,12 @@
       </c>
       <c r="B106" s="10" t="inlineStr">
         <is>
-          <t>Home</t>
+          <t>Authentication</t>
         </is>
       </c>
       <c r="C106" s="10" t="inlineStr">
         <is>
-          <t>Automated Mobile Test Case Detail #99</t>
+          <t>Verify In-App Banner Alerts System Notifications</t>
         </is>
       </c>
       <c r="D106" s="11" t="inlineStr">
@@ -3902,12 +3902,12 @@
       </c>
       <c r="E106" s="10" t="inlineStr">
         <is>
-          <t>899 ms</t>
+          <t>181 ms</t>
         </is>
       </c>
       <c r="F106" s="10" t="inlineStr">
         <is>
-          <t>2026-06-17 10:38:10</t>
+          <t>2026-06-17 10:47:04</t>
         </is>
       </c>
       <c r="G106" s="10" t="inlineStr"/>
@@ -3920,12 +3920,12 @@
       </c>
       <c r="B107" s="12" t="inlineStr">
         <is>
-          <t>Marketplace</t>
+          <t>Home</t>
         </is>
       </c>
       <c r="C107" s="12" t="inlineStr">
         <is>
-          <t>Automated Mobile Test Case Detail #100</t>
+          <t>Check App Launch Update Check Version Modal</t>
         </is>
       </c>
       <c r="D107" s="11" t="inlineStr">
@@ -3935,12 +3935,12 @@
       </c>
       <c r="E107" s="12" t="inlineStr">
         <is>
-          <t>320 ms</t>
+          <t>679 ms</t>
         </is>
       </c>
       <c r="F107" s="12" t="inlineStr">
         <is>
-          <t>2026-06-17 10:38:10</t>
+          <t>2026-06-17 10:47:04</t>
         </is>
       </c>
       <c r="G107" s="12" t="inlineStr"/>
@@ -3953,12 +3953,12 @@
       </c>
       <c r="B108" s="10" t="inlineStr">
         <is>
-          <t>Sell</t>
+          <t>Marketplace</t>
         </is>
       </c>
       <c r="C108" s="10" t="inlineStr">
         <is>
-          <t>Automated Mobile Test Case Detail #101</t>
+          <t>Verify App Store Redirect Button Version Check</t>
         </is>
       </c>
       <c r="D108" s="11" t="inlineStr">
@@ -3968,12 +3968,12 @@
       </c>
       <c r="E108" s="10" t="inlineStr">
         <is>
-          <t>425 ms</t>
+          <t>802 ms</t>
         </is>
       </c>
       <c r="F108" s="10" t="inlineStr">
         <is>
-          <t>2026-06-17 10:38:10</t>
+          <t>2026-06-17 10:47:04</t>
         </is>
       </c>
       <c r="G108" s="10" t="inlineStr"/>
@@ -3986,12 +3986,12 @@
       </c>
       <c r="B109" s="12" t="inlineStr">
         <is>
-          <t>Profile</t>
+          <t>Sell</t>
         </is>
       </c>
       <c r="C109" s="12" t="inlineStr">
         <is>
-          <t>Automated Mobile Test Case Detail #102</t>
+          <t>Verify System Crash Error Boundary Recovery</t>
         </is>
       </c>
       <c r="D109" s="11" t="inlineStr">
@@ -4001,12 +4001,12 @@
       </c>
       <c r="E109" s="12" t="inlineStr">
         <is>
-          <t>872 ms</t>
+          <t>219 ms</t>
         </is>
       </c>
       <c r="F109" s="12" t="inlineStr">
         <is>
-          <t>2026-06-17 10:38:10</t>
+          <t>2026-06-17 10:47:04</t>
         </is>
       </c>
       <c r="G109" s="12" t="inlineStr"/>
@@ -4019,12 +4019,12 @@
       </c>
       <c r="B110" s="10" t="inlineStr">
         <is>
-          <t>Chat</t>
+          <t>Profile</t>
         </is>
       </c>
       <c r="C110" s="10" t="inlineStr">
         <is>
-          <t>Automated Mobile Test Case Detail #103</t>
+          <t>Verify Network Timeout Warning Alert Banner</t>
         </is>
       </c>
       <c r="D110" s="11" t="inlineStr">
@@ -4034,12 +4034,12 @@
       </c>
       <c r="E110" s="10" t="inlineStr">
         <is>
-          <t>176 ms</t>
+          <t>791 ms</t>
         </is>
       </c>
       <c r="F110" s="10" t="inlineStr">
         <is>
-          <t>2026-06-17 10:38:10</t>
+          <t>2026-06-17 10:47:04</t>
         </is>
       </c>
       <c r="G110" s="10" t="inlineStr"/>
@@ -4052,12 +4052,12 @@
       </c>
       <c r="B111" s="12" t="inlineStr">
         <is>
-          <t>Settings</t>
+          <t>Chat</t>
         </is>
       </c>
       <c r="C111" s="12" t="inlineStr">
         <is>
-          <t>Automated Mobile Test Case Detail #104</t>
+          <t>Check App Performance Memory Usage Benchmarks</t>
         </is>
       </c>
       <c r="D111" s="11" t="inlineStr">
@@ -4067,12 +4067,12 @@
       </c>
       <c r="E111" s="12" t="inlineStr">
         <is>
-          <t>859 ms</t>
+          <t>143 ms</t>
         </is>
       </c>
       <c r="F111" s="12" t="inlineStr">
         <is>
-          <t>2026-06-17 10:38:10</t>
+          <t>2026-06-17 10:47:04</t>
         </is>
       </c>
       <c r="G111" s="12" t="inlineStr"/>
@@ -4085,12 +4085,12 @@
       </c>
       <c r="B112" s="10" t="inlineStr">
         <is>
-          <t>Authentication</t>
+          <t>Settings</t>
         </is>
       </c>
       <c r="C112" s="10" t="inlineStr">
         <is>
-          <t>Automated Mobile Test Case Detail #105</t>
+          <t>Verify App Battery Drain Minimization Standards</t>
         </is>
       </c>
       <c r="D112" s="11" t="inlineStr">
@@ -4100,12 +4100,12 @@
       </c>
       <c r="E112" s="10" t="inlineStr">
         <is>
-          <t>831 ms</t>
+          <t>618 ms</t>
         </is>
       </c>
       <c r="F112" s="10" t="inlineStr">
         <is>
-          <t>2026-06-17 10:38:10</t>
+          <t>2026-06-17 10:47:04</t>
         </is>
       </c>
       <c r="G112" s="10" t="inlineStr"/>

</xml_diff>